<commit_message>
Update binary content of transactions Excel file to reflect the latest changes in data
</commit_message>
<xml_diff>
--- a/data/transactions/أذونات الإضافة لشهر 4.xlsx
+++ b/data/transactions/أذونات الإضافة لشهر 4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ERP\erp-server\data\transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F65D7D5-9544-46B1-ABD1-6F640C9A6C60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B84CEE0-496E-41FB-A451-09DA047A29C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="977" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="978" uniqueCount="414">
   <si>
     <t>م</t>
   </si>
@@ -1474,7 +1474,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1522,6 +1522,15 @@
     </xf>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3588,10 +3597,18 @@
       <c r="C50" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="D50" s="20"/>
-      <c r="E50" s="19"/>
-      <c r="F50" s="19"/>
-      <c r="G50" s="19"/>
+      <c r="D50" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="E50" s="19">
+        <v>2050</v>
+      </c>
+      <c r="F50" s="19">
+        <v>35.979999999999997</v>
+      </c>
+      <c r="G50" s="19">
+        <v>73759</v>
+      </c>
       <c r="H50" s="3">
         <v>705</v>
       </c>
@@ -3619,16 +3636,16 @@
       <c r="C51" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D51" s="20" t="s">
+      <c r="D51" s="23" t="s">
         <v>83</v>
       </c>
-      <c r="E51" s="18">
+      <c r="E51" s="21">
         <v>430</v>
       </c>
-      <c r="F51" s="18">
+      <c r="F51" s="21">
         <v>50.88</v>
       </c>
-      <c r="G51" s="18">
+      <c r="G51" s="21">
         <v>21319.599999999999</v>
       </c>
       <c r="H51" s="3">
@@ -3658,10 +3675,10 @@
       <c r="C52" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="D52" s="19"/>
-      <c r="E52" s="19"/>
-      <c r="F52" s="19"/>
-      <c r="G52" s="19"/>
+      <c r="D52" s="22"/>
+      <c r="E52" s="22"/>
+      <c r="F52" s="22"/>
+      <c r="G52" s="22"/>
       <c r="H52" s="3">
         <v>705</v>
       </c>
@@ -9302,15 +9319,11 @@
     </row>
     <row r="198" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="G49:G50"/>
+  <mergeCells count="4">
     <mergeCell ref="F51:F52"/>
     <mergeCell ref="G51:G52"/>
-    <mergeCell ref="D49:D50"/>
     <mergeCell ref="D51:D52"/>
-    <mergeCell ref="E49:E50"/>
     <mergeCell ref="E51:E52"/>
-    <mergeCell ref="F49:F50"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>

<commit_message>
Update Excel transaction file with new data
</commit_message>
<xml_diff>
--- a/data/transactions/أذونات الإضافة لشهر 4.xlsx
+++ b/data/transactions/أذونات الإضافة لشهر 4.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ERP\erp-server\data\transactions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ERP\Development\erp-server\data\transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B84CEE0-496E-41FB-A451-09DA047A29C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D88FB4E-013E-497B-A673-D163FD7A52D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1833,7 +1833,7 @@
     <col min="7" max="7" width="15.28515625" customWidth="1"/>
     <col min="8" max="8" width="13.28515625" customWidth="1"/>
     <col min="9" max="10" width="18.7109375" customWidth="1"/>
-    <col min="11" max="11" width="23.140625" customWidth="1"/>
+    <col min="11" max="11" width="26.5703125" customWidth="1"/>
     <col min="12" max="12" width="14.85546875" customWidth="1"/>
     <col min="13" max="13" width="15.140625" customWidth="1"/>
   </cols>
@@ -3867,10 +3867,10 @@
         <v>2105</v>
       </c>
       <c r="F57" s="5">
-        <v>153508.76999999999</v>
+        <v>153.50877</v>
       </c>
       <c r="G57" s="3">
-        <v>1123135.96</v>
+        <v>323136.44500000001</v>
       </c>
       <c r="H57" s="3">
         <v>59809</v>

</xml_diff>

<commit_message>
Update Excel transaction files 3 and 4 with new revisions
</commit_message>
<xml_diff>
--- a/data/transactions/أذونات الإضافة لشهر 4.xlsx
+++ b/data/transactions/أذونات الإضافة لشهر 4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ERP\Development\erp-server\data\transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D88FB4E-013E-497B-A673-D163FD7A52D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D51BE915-5690-4C39-BB62-BEB1520CA2FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,10 +18,19 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$M$197</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -31,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="978" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="979" uniqueCount="414">
   <si>
     <t>م</t>
   </si>
@@ -1474,7 +1483,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1533,9 +1542,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1826,7 +1832,7 @@
   <cols>
     <col min="1" max="1" width="6.5703125" customWidth="1"/>
     <col min="2" max="2" width="16.5703125" customWidth="1"/>
-    <col min="3" max="3" width="31.28515625" customWidth="1"/>
+    <col min="3" max="3" width="53.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.140625" customWidth="1"/>
     <col min="5" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.85546875" customWidth="1"/>
@@ -1834,7 +1840,7 @@
     <col min="8" max="8" width="13.28515625" customWidth="1"/>
     <col min="9" max="10" width="18.7109375" customWidth="1"/>
     <col min="11" max="11" width="26.5703125" customWidth="1"/>
-    <col min="12" max="12" width="14.85546875" customWidth="1"/>
+    <col min="12" max="12" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3562,13 +3568,14 @@
         <v>83</v>
       </c>
       <c r="E49" s="18">
-        <v>2050</v>
+        <v>1022</v>
       </c>
       <c r="F49" s="18">
         <v>35.979999999999997</v>
       </c>
       <c r="G49" s="18">
-        <v>73759</v>
+        <f>E49*F49</f>
+        <v>36771.56</v>
       </c>
       <c r="H49" s="3">
         <v>705</v>
@@ -3601,13 +3608,14 @@
         <v>83</v>
       </c>
       <c r="E50" s="19">
-        <v>2050</v>
+        <v>942</v>
       </c>
       <c r="F50" s="19">
         <v>35.979999999999997</v>
       </c>
-      <c r="G50" s="19">
-        <v>73759</v>
+      <c r="G50" s="21">
+        <f t="shared" ref="G50:G52" si="0">E50*F50</f>
+        <v>33893.159999999996</v>
       </c>
       <c r="H50" s="3">
         <v>705</v>
@@ -3636,17 +3644,18 @@
       <c r="C51" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D51" s="23" t="s">
+      <c r="D51" s="22" t="s">
         <v>83</v>
       </c>
       <c r="E51" s="21">
-        <v>430</v>
+        <v>374.1</v>
       </c>
       <c r="F51" s="21">
         <v>50.88</v>
       </c>
       <c r="G51" s="21">
-        <v>21319.599999999999</v>
+        <f t="shared" si="0"/>
+        <v>19034.208000000002</v>
       </c>
       <c r="H51" s="3">
         <v>705</v>
@@ -3675,10 +3684,19 @@
       <c r="C52" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="D52" s="22"/>
-      <c r="E52" s="22"/>
-      <c r="F52" s="22"/>
-      <c r="G52" s="22"/>
+      <c r="D52" s="22" t="s">
+        <v>83</v>
+      </c>
+      <c r="E52" s="21">
+        <v>141.30000000000001</v>
+      </c>
+      <c r="F52" s="21">
+        <v>50.88</v>
+      </c>
+      <c r="G52" s="21">
+        <f t="shared" si="0"/>
+        <v>7189.344000000001</v>
+      </c>
       <c r="H52" s="3">
         <v>705</v>
       </c>
@@ -9319,12 +9337,6 @@
     </row>
     <row r="198" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="F51:F52"/>
-    <mergeCell ref="G51:G52"/>
-    <mergeCell ref="D51:D52"/>
-    <mergeCell ref="E51:E52"/>
-  </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update transaction Excel files with new data revisions for files 4 and 5
</commit_message>
<xml_diff>
--- a/data/transactions/أذونات الإضافة لشهر 4.xlsx
+++ b/data/transactions/أذونات الإضافة لشهر 4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ERP\Development\erp-server\data\transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D51BE915-5690-4C39-BB62-BEB1520CA2FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE477839-A327-4D8D-B01E-DAA02F45680C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3169,7 +3169,7 @@
         <v>33</v>
       </c>
       <c r="B39" s="5">
-        <v>1105001</v>
+        <v>11105001</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>72</v>
@@ -3918,12 +3918,14 @@
         <v>94</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>13</v>
+        <v>83</v>
       </c>
       <c r="E58" s="3">
-        <v>133</v>
-      </c>
-      <c r="F58" s="3"/>
+        <v>1702.4</v>
+      </c>
+      <c r="F58" s="3">
+        <v>45.61</v>
+      </c>
       <c r="G58" s="3">
         <v>90079.75</v>
       </c>

</xml_diff>